<commit_message>
fixing symbol of thermodyn temperature
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Notes.xlsx
+++ b/CUQ/_docs/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gruber04\git_repos\BIPM\Semantic-SI\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6E7C8C-F8F3-4836-B380-1BEE1E4BE94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5E0589-6050-4105-971C-A724E96B92BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-8310" windowWidth="38640" windowHeight="21390" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1961,104 +1961,104 @@
     <t>\rm{T}</t>
   </si>
   <si>
-    <t>As a result of the way temperature scales used to be defined, it remains common practice to express a thermodynamic temperature, symbol @kels@, in terms of its difference from the reference temperature @fpwd@, close to the ice point. This difference is called the Celsius temperature, symbol @cels@ which is defined by the quantity equation \[@celd@\].</t>
-  </si>
-  <si>
-    <t>En raison de la manière dont les échelles de température étaient habituellement définies, il est resté d’usage courant d’exprimer la température thermodynamique, symbole @kels@, en fonction de sa différence par rapport à la température de référence @fpwd@ proche du point de congélation de l’eau. Cette différence de température est appelée température Celsius, symbole @cels@ ; elle est définie par l’équation aux grandeurs :
+    <t>\rm{@circ@{C}}</t>
+  </si>
+  <si>
+    <t>ITS-90 Celsius symbol</t>
+  </si>
+  <si>
+    <t>Celsius to Kelvin definition</t>
+  </si>
+  <si>
+    <t>Inverse Celsius to Kelvin offset (French)</t>
+  </si>
+  <si>
+    <t>Celsius to Kelvin offset (French)</t>
+  </si>
+  <si>
+    <t>Celsius temperature quantity definition</t>
+  </si>
+  <si>
+    <t>Celsius temperature quantity equation</t>
+  </si>
+  <si>
+    <t>Inverse Celsius to Kelvin offset (English)</t>
+  </si>
+  <si>
+    <t>Celsius to Kelvin offset (English)</t>
+  </si>
+  <si>
+    <t>Celsius temperature quantity symbol</t>
+  </si>
+  <si>
+    <t>Celsius unit symbol</t>
+  </si>
+  <si>
+    <t>Boltzmann constant / (Planck constant *elementary charge) value</t>
+  </si>
+  <si>
+    <t>Hyperfine caesium constant symbol</t>
+  </si>
+  <si>
+    <t>Hyperfine caesium constant unit</t>
+  </si>
+  <si>
+    <t>Hyperfine caesium constant value</t>
+  </si>
+  <si>
+    <t>Hyperfine caesium constant exact relation</t>
+  </si>
+  <si>
+    <t>Hyperfine caesium/speed of light value</t>
+  </si>
+  <si>
+    <t>Inverse hyperfine caesium elementary charge value</t>
+  </si>
+  <si>
+    <t>Candela steradian per kilogram inv. metre squared. second cubed unit symbol</t>
+  </si>
+  <si>
+    <t>Kilogram, metre squared, inverse second squared, per kelvin unit symbol</t>
+  </si>
+  <si>
+    <t>Kilogram, metre squared, inverse second unit symbol</t>
+  </si>
+  <si>
+    <t>Kilogram metre squared second inv. squared per kelvin unit symbol</t>
+  </si>
+  <si>
+    <t>Per square metre second unit symbol</t>
+  </si>
+  <si>
+    <t>Radiation direction value/unit</t>
+  </si>
+  <si>
+    <t>Caesium 133 isotope symbol</t>
+  </si>
+  <si>
+    <t>Metre horizontal plane distance value/unit</t>
+  </si>
+  <si>
+    <t>Metre unit definition</t>
+  </si>
+  <si>
+    <t>Metre unit symbol</t>
+  </si>
+  <si>
+    <t>Metre vacuum wavelengths value</t>
+  </si>
+  <si>
+    <t>Molar mass via Avogadro constant definition</t>
+  </si>
+  <si>
+    <t>Note that with the present definition, primary realizations of the kelvin can, in principle, be established at any point of the temperature scale.</t>
+  </si>
+  <si>
+    <t>As a result of the way temperature scales used to be defined, it remains common practice to express a thermodynamic temperature, symbol @tmps@, in terms of its difference from the reference temperature @fpwd@, close to the ice point. This difference is called the Celsius temperature, symbol @cels@ which is defined by the quantity equation \[@celd@\].</t>
+  </si>
+  <si>
+    <t>En raison de la manière dont les échelles de température étaient habituellement définies, il est resté d’usage courant d’exprimer la température thermodynamique, symbole @tmps@, en fonction de sa différence par rapport à la température de référence @fpwd@ proche du point de congélation de l’eau. Cette différence de température est appelée température Celsius, symbole @cels@ ; elle est définie par l’équation aux grandeurs :
 \[@celd@\].</t>
-  </si>
-  <si>
-    <t>\rm{@circ@{C}}</t>
-  </si>
-  <si>
-    <t>ITS-90 Celsius symbol</t>
-  </si>
-  <si>
-    <t>Celsius to Kelvin definition</t>
-  </si>
-  <si>
-    <t>Inverse Celsius to Kelvin offset (French)</t>
-  </si>
-  <si>
-    <t>Celsius to Kelvin offset (French)</t>
-  </si>
-  <si>
-    <t>Celsius temperature quantity definition</t>
-  </si>
-  <si>
-    <t>Celsius temperature quantity equation</t>
-  </si>
-  <si>
-    <t>Inverse Celsius to Kelvin offset (English)</t>
-  </si>
-  <si>
-    <t>Celsius to Kelvin offset (English)</t>
-  </si>
-  <si>
-    <t>Celsius temperature quantity symbol</t>
-  </si>
-  <si>
-    <t>Celsius unit symbol</t>
-  </si>
-  <si>
-    <t>Boltzmann constant / (Planck constant *elementary charge) value</t>
-  </si>
-  <si>
-    <t>Hyperfine caesium constant symbol</t>
-  </si>
-  <si>
-    <t>Hyperfine caesium constant unit</t>
-  </si>
-  <si>
-    <t>Hyperfine caesium constant value</t>
-  </si>
-  <si>
-    <t>Hyperfine caesium constant exact relation</t>
-  </si>
-  <si>
-    <t>Hyperfine caesium/speed of light value</t>
-  </si>
-  <si>
-    <t>Inverse hyperfine caesium elementary charge value</t>
-  </si>
-  <si>
-    <t>Candela steradian per kilogram inv. metre squared. second cubed unit symbol</t>
-  </si>
-  <si>
-    <t>Kilogram, metre squared, inverse second squared, per kelvin unit symbol</t>
-  </si>
-  <si>
-    <t>Kilogram, metre squared, inverse second unit symbol</t>
-  </si>
-  <si>
-    <t>Kilogram metre squared second inv. squared per kelvin unit symbol</t>
-  </si>
-  <si>
-    <t>Per square metre second unit symbol</t>
-  </si>
-  <si>
-    <t>Radiation direction value/unit</t>
-  </si>
-  <si>
-    <t>Caesium 133 isotope symbol</t>
-  </si>
-  <si>
-    <t>Metre horizontal plane distance value/unit</t>
-  </si>
-  <si>
-    <t>Metre unit definition</t>
-  </si>
-  <si>
-    <t>Metre unit symbol</t>
-  </si>
-  <si>
-    <t>Metre vacuum wavelengths value</t>
-  </si>
-  <si>
-    <t>Molar mass via Avogadro constant definition</t>
-  </si>
-  <si>
-    <t>Note that with the present definition, primary realizations of the kelvin can, in principle, be established at any point of the temperature scale.</t>
   </si>
 </sst>
 </file>
@@ -3313,7 +3313,7 @@
         <v>4</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>640</v>
+        <v>671</v>
       </c>
       <c r="E21" s="4">
         <v>44978.666134259256</v>
@@ -3364,7 +3364,7 @@
         <v>7</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="E24" s="4">
         <v>44978.666134259256</v>
@@ -4286,7 +4286,7 @@
         <v>4</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>641</v>
+        <v>672</v>
       </c>
     </row>
     <row r="22" spans="1:4" s="2" customFormat="1" ht="78.75">
@@ -4910,7 +4910,7 @@
         <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
@@ -5231,7 +5231,7 @@
         <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D20" t="s">
         <v>38</v>
@@ -5248,7 +5248,7 @@
         <v>65</v>
       </c>
       <c r="B21" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="D21" t="s">
         <v>78</v>
@@ -5316,7 +5316,7 @@
         <v>134</v>
       </c>
       <c r="B25" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="D25" t="s">
         <v>38</v>
@@ -5333,7 +5333,7 @@
         <v>133</v>
       </c>
       <c r="B26" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="D26" t="s">
         <v>38</v>
@@ -5350,7 +5350,7 @@
         <v>63</v>
       </c>
       <c r="B27" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="D27" t="s">
         <v>78</v>
@@ -5367,7 +5367,7 @@
         <v>91</v>
       </c>
       <c r="B28" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D28" t="s">
         <v>78</v>
@@ -5384,7 +5384,7 @@
         <v>135</v>
       </c>
       <c r="B29" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="D29" t="s">
         <v>38</v>
@@ -5401,7 +5401,7 @@
         <v>113</v>
       </c>
       <c r="B30" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D30" t="s">
         <v>38</v>
@@ -5418,7 +5418,7 @@
         <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D31" t="s">
         <v>38</v>
@@ -5435,7 +5435,7 @@
         <v>64</v>
       </c>
       <c r="B32" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D32" t="s">
         <v>38</v>
@@ -5444,7 +5444,7 @@
         <v>233</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -5509,7 +5509,7 @@
         <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -5526,7 +5526,7 @@
         <v>122</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="D37" t="s">
         <v>38</v>
@@ -5560,7 +5560,7 @@
         <v>88</v>
       </c>
       <c r="B39" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D39" t="s">
         <v>38</v>
@@ -5892,7 +5892,7 @@
         <v>4</v>
       </c>
       <c r="B58" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D58" t="s">
         <v>38</v>
@@ -5918,7 +5918,7 @@
         <v>89</v>
       </c>
       <c r="B59" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D59" t="s">
         <v>38</v>
@@ -5935,7 +5935,7 @@
         <v>14</v>
       </c>
       <c r="B60" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D60" t="s">
         <v>38</v>
@@ -5961,7 +5961,7 @@
         <v>31</v>
       </c>
       <c r="B61" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D61" t="s">
         <v>38</v>
@@ -5978,7 +5978,7 @@
         <v>15</v>
       </c>
       <c r="B62" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D62" t="s">
         <v>38</v>
@@ -6004,7 +6004,7 @@
         <v>108</v>
       </c>
       <c r="B63" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D63" t="s">
         <v>38</v>
@@ -6202,7 +6202,7 @@
         <v>124</v>
       </c>
       <c r="B72" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D72" t="s">
         <v>38</v>
@@ -6236,7 +6236,7 @@
         <v>125</v>
       </c>
       <c r="B74" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D74" t="s">
         <v>38</v>
@@ -6253,7 +6253,7 @@
         <v>109</v>
       </c>
       <c r="B75" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D75" t="s">
         <v>38</v>
@@ -6409,7 +6409,7 @@
         <v>81</v>
       </c>
       <c r="B84" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="D84" t="s">
         <v>78</v>
@@ -6647,7 +6647,7 @@
         <v>126</v>
       </c>
       <c r="B98" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="D98" t="s">
         <v>38</v>
@@ -6664,7 +6664,7 @@
         <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D99" t="s">
         <v>78</v>
@@ -6690,7 +6690,7 @@
         <v>5</v>
       </c>
       <c r="B100" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="D100" t="s">
         <v>38</v>
@@ -6716,7 +6716,7 @@
         <v>127</v>
       </c>
       <c r="B101" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D101" t="s">
         <v>38</v>
@@ -7111,7 +7111,7 @@
         <v>24</v>
       </c>
       <c r="B120" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D120" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Fix errors in excel files
- n -> "Luminous Efficacy" for candela1979 in Units_Prefixes.xls
- blank cells -> 1 / No note for candela1979 in Notes.xls

Final (?) changes before ditching xlsx files ?
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Notes.xlsx
+++ b/CUQ/_docs/Notes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gruber04\git_repos\BIPM\Semantic-SI\CUQ\_docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\fmeynadier\git_projects\SI-Reference-Point-2023\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FAF9511-BE2B-4822-A852-96CD9A0C43CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DABC3E-DC47-43F4-A646-CA2F228465B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-8310" windowWidth="38640" windowHeight="21390" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="2265" windowWidth="23325" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="en" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="673">
   <si>
     <t>id</t>
   </si>
@@ -2692,48 +2692,48 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Akzent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Akzent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Akzent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Akzent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Akzent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Akzent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Ausgabe" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Berechnung" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Eingabe" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Überschrift 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Warnender Text" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20 % - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20 % - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20 % - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20 % - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20 % - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40 % - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40 % - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40 % - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40 % - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40 % - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40 % - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60 % - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60 % - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60 % - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60 % - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60 % - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60 % - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Avertissement" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Calcul" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Cellule liée" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Entrée" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Insatisfaisant" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Neutre" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Satisfaisant" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Sortie" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texte explicatif" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Titre" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Titre 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Titre 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Titre 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Titre 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Vérification" xfId="13" builtinId="23" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2754,7 +2754,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -4817,7 +4817,12 @@
       <c r="B54" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="D54" s="10"/>
+      <c r="C54" s="8">
+        <v>1</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>509</v>
+      </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="3">
@@ -4959,6 +4964,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added "No notes" for candela1979 to avoid None
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Notes.xlsx
+++ b/CUQ/_docs/Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\fmeynadier\git_projects\SI-Reference-Point-2023\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DABC3E-DC47-43F4-A646-CA2F228465B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8373D1A5-9029-470B-AB07-1EE3A80F6201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="2265" windowWidth="23325" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5445" yWindow="1890" windowWidth="23325" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="en" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="673">
   <si>
     <t>id</t>
   </si>
@@ -2147,7 +2147,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2301,10 +2301,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="TimesNewRomanPSMT"/>
     </font>
     <font>
       <sz val="9"/>
@@ -2663,7 +2659,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2684,12 +2680,11 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="22" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3051,7 +3046,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E62"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5" style="8" customWidth="1"/>
     <col min="2" max="2" width="16.875" style="8" customWidth="1"/>
@@ -3061,7 +3056,7 @@
     <col min="6" max="16384" width="11" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>342</v>
       </c>
@@ -3078,7 +3073,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="3" customFormat="1">
+    <row r="2" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -3095,7 +3090,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="3" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -3112,7 +3107,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="4" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -3129,7 +3124,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="5" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -3146,7 +3141,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="6" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -3163,7 +3158,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="3" customFormat="1">
+    <row r="7" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -3180,7 +3175,7 @@
         <v>45104.336331018516</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="3" customFormat="1">
+    <row r="8" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -3197,7 +3192,7 @@
         <v>45104.365567129629</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="9" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -3214,7 +3209,7 @@
         <v>45105.140208333331</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="10" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -3231,7 +3226,7 @@
         <v>45105.154224537036</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="11" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -3248,7 +3243,7 @@
         <v>45105.16302083333</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="3" customFormat="1">
+    <row r="12" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -3265,7 +3260,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="13" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -3282,7 +3277,7 @@
         <v>45105.158726851849</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="14" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -3299,7 +3294,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="3" customFormat="1">
+    <row r="15" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -3316,7 +3311,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="3" customFormat="1" ht="47.25">
+    <row r="16" spans="1:5" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -3333,7 +3328,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="3" customFormat="1" ht="63">
+    <row r="17" spans="1:5" s="3" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -3350,7 +3345,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="18" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -3367,7 +3362,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="3" customFormat="1">
+    <row r="19" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -3384,7 +3379,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="3" customFormat="1" ht="47.25">
+    <row r="20" spans="1:5" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -3401,7 +3396,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="21" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -3418,7 +3413,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="3" customFormat="1" ht="47.25">
+    <row r="22" spans="1:5" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -3435,7 +3430,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="23" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -3452,7 +3447,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="3" customFormat="1">
+    <row r="24" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -3469,7 +3464,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="3" customFormat="1">
+    <row r="25" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -3486,7 +3481,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="3" customFormat="1">
+    <row r="26" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -3503,7 +3498,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="3" customFormat="1" ht="47.25">
+    <row r="27" spans="1:5" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -3520,7 +3515,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="28" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -3537,7 +3532,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="29" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -3554,7 +3549,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="3" customFormat="1" ht="78.75">
+    <row r="30" spans="1:5" s="3" customFormat="1" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -3571,7 +3566,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="31" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -3588,7 +3583,7 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="32" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -3605,7 +3600,7 @@
         <v>44944.721134259256</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="3" customFormat="1">
+    <row r="33" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -3622,7 +3617,7 @@
         <v>44944.729699074072</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="3" customFormat="1">
+    <row r="34" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -3639,7 +3634,7 @@
         <v>44944.729988425926</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="3" customFormat="1">
+    <row r="35" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -3656,7 +3651,7 @@
         <v>44944.728692129633</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="3" customFormat="1">
+    <row r="36" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -3673,7 +3668,7 @@
         <v>44944.730671296296</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="3" customFormat="1">
+    <row r="37" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -3690,7 +3685,7 @@
         <v>44944.731365740743</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="3" customFormat="1">
+    <row r="38" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -3707,7 +3702,7 @@
         <v>44944.731944444444</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="3" customFormat="1">
+    <row r="39" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -3724,7 +3719,7 @@
         <v>44944.732581018521</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="3" customFormat="1">
+    <row r="40" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -3741,7 +3736,7 @@
         <v>44944.732546296298</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="3" customFormat="1">
+    <row r="41" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -3758,7 +3753,7 @@
         <v>44944.729699074072</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="3" customFormat="1">
+    <row r="42" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -3775,7 +3770,7 @@
         <v>44944.729699074072</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="3" customFormat="1">
+    <row r="43" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -3792,7 +3787,7 @@
         <v>44944.728715277779</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="3" customFormat="1">
+    <row r="44" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -3809,7 +3804,7 @@
         <v>44944.72865740741</v>
       </c>
     </row>
-    <row r="45" spans="1:5" s="3" customFormat="1">
+    <row r="45" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -3826,7 +3821,7 @@
         <v>44944.728634259256</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="3" customFormat="1">
+    <row r="46" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -3843,7 +3838,7 @@
         <v>44944.732604166667</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="3" customFormat="1">
+    <row r="47" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -3860,7 +3855,7 @@
         <v>44944.732523148145</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="3" customFormat="1">
+    <row r="48" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -3877,7 +3872,7 @@
         <v>44944.731400462966</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="3" customFormat="1" ht="17.100000000000001" customHeight="1">
+    <row r="49" spans="1:5" s="3" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -3894,7 +3889,7 @@
         <v>44944.73133101852</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="3" customFormat="1">
+    <row r="50" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -3911,10 +3906,10 @@
         <v>44978.666134259256</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B51" s="7"/>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>50</v>
       </c>
@@ -3931,16 +3926,21 @@
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>51</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="D54" s="10"/>
-    </row>
-    <row r="55" spans="1:5">
+      <c r="C54" s="8">
+        <v>1</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>52</v>
       </c>
@@ -3957,7 +3957,7 @@
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="47.25">
+    <row r="56" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>53</v>
       </c>
@@ -3967,14 +3967,14 @@
       <c r="C56" s="3">
         <v>2</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="10" t="s">
         <v>658</v>
       </c>
       <c r="E56" s="6">
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>54</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>55</v>
       </c>
@@ -4001,14 +4001,14 @@
       <c r="C58" s="3">
         <v>1</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="10" t="s">
         <v>514</v>
       </c>
       <c r="E58" s="6">
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>56</v>
       </c>
@@ -4018,14 +4018,14 @@
       <c r="C59" s="3">
         <v>1</v>
       </c>
-      <c r="D59" s="11" t="s">
+      <c r="D59" s="10" t="s">
         <v>514</v>
       </c>
       <c r="E59" s="6">
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>57</v>
       </c>
@@ -4042,7 +4042,7 @@
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -4059,7 +4059,7 @@
         <v>45126.62222222222</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>59</v>
       </c>
@@ -4085,7 +4085,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C76578C5-08B3-574F-BA8C-FE251C939966}">
   <dimension ref="A1:E70"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5" style="8" customWidth="1"/>
     <col min="2" max="2" width="14.5" style="8" customWidth="1"/>
@@ -4095,7 +4095,7 @@
     <col min="6" max="16384" width="11" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="3" customFormat="1">
+    <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -4123,7 +4123,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="3" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -4137,7 +4137,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="4" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -4151,7 +4151,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="5" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -4165,7 +4165,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="3" customFormat="1" ht="47.25">
+    <row r="6" spans="1:4" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -4179,7 +4179,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="3" customFormat="1">
+    <row r="7" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="3" customFormat="1">
+    <row r="8" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="9" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -4221,7 +4221,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="10" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -4235,7 +4235,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="11" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="3" customFormat="1">
+    <row r="12" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -4263,7 +4263,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="3" customFormat="1" ht="47.25">
+    <row r="13" spans="1:4" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -4277,7 +4277,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="14" spans="1:4" s="3" customFormat="1">
+    <row r="14" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -4291,7 +4291,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="15" spans="1:4" s="3" customFormat="1">
+    <row r="15" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="16" spans="1:4" s="3" customFormat="1" ht="47.25">
+    <row r="16" spans="1:4" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -4319,7 +4319,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="17" spans="1:4" s="3" customFormat="1" ht="63">
+    <row r="17" spans="1:4" s="3" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -4333,7 +4333,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="18" spans="1:4" s="3" customFormat="1">
+    <row r="18" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="19" spans="1:4" s="3" customFormat="1">
+    <row r="19" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -4361,7 +4361,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="20" spans="1:4" s="3" customFormat="1" ht="47.25">
+    <row r="20" spans="1:4" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -4375,7 +4375,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="21" spans="1:4" s="3" customFormat="1" ht="63">
+    <row r="21" spans="1:4" s="3" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="22" spans="1:4" s="3" customFormat="1" ht="63">
+    <row r="22" spans="1:4" s="3" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="23" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="23" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="24" spans="1:4" s="3" customFormat="1">
+    <row r="24" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -4431,7 +4431,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="25" spans="1:4" s="3" customFormat="1">
+    <row r="25" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -4445,7 +4445,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="26" spans="1:4" s="3" customFormat="1">
+    <row r="26" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="27" spans="1:4" s="3" customFormat="1" ht="47.25">
+    <row r="27" spans="1:4" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -4473,7 +4473,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="28" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="28" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -4487,7 +4487,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="29" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="29" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -4501,7 +4501,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="30" spans="1:4" s="3" customFormat="1" ht="78.75">
+    <row r="30" spans="1:4" s="3" customFormat="1" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="31" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="31" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="32" spans="1:4" s="3" customFormat="1" ht="31.5">
+    <row r="32" spans="1:4" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -4543,7 +4543,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="33" spans="1:4" s="3" customFormat="1">
+    <row r="33" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -4557,7 +4557,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="34" spans="1:4" s="3" customFormat="1">
+    <row r="34" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -4571,7 +4571,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="35" spans="1:4" s="3" customFormat="1">
+    <row r="35" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -4585,7 +4585,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="36" spans="1:4" s="3" customFormat="1">
+    <row r="36" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="37" spans="1:4" s="3" customFormat="1">
+    <row r="37" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -4613,7 +4613,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="38" spans="1:4" s="3" customFormat="1">
+    <row r="38" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -4627,7 +4627,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="39" spans="1:4" s="3" customFormat="1">
+    <row r="39" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -4641,7 +4641,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="40" spans="1:4" s="3" customFormat="1">
+    <row r="40" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -4655,7 +4655,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="41" spans="1:4" s="3" customFormat="1">
+    <row r="41" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>51</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="42" spans="1:4" s="3" customFormat="1">
+    <row r="42" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>52</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="43" spans="1:4" s="3" customFormat="1">
+    <row r="43" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>53</v>
       </c>
@@ -4697,7 +4697,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="44" spans="1:4" s="3" customFormat="1">
+    <row r="44" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>54</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="45" spans="1:4" s="3" customFormat="1">
+    <row r="45" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>55</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="46" spans="1:4" s="3" customFormat="1">
+    <row r="46" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>56</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="47" spans="1:4" s="3" customFormat="1">
+    <row r="47" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>57</v>
       </c>
@@ -4753,7 +4753,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="48" spans="1:4" s="3" customFormat="1">
+    <row r="48" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>58</v>
       </c>
@@ -4767,7 +4767,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="3" customFormat="1" ht="17.100000000000001" customHeight="1">
+    <row r="49" spans="1:5" s="3" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>59</v>
       </c>
@@ -4781,7 +4781,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="3" customFormat="1" ht="31.5">
+    <row r="50" spans="1:5" s="3" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>70</v>
       </c>
@@ -4795,7 +4795,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>50</v>
       </c>
@@ -4810,7 +4810,7 @@
       </c>
       <c r="E53" s="9"/>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>51</v>
       </c>
@@ -4824,7 +4824,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>52</v>
       </c>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E55" s="9"/>
     </row>
-    <row r="56" spans="1:5" ht="47.25">
+    <row r="56" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>53</v>
       </c>
@@ -4849,12 +4849,12 @@
       <c r="C56" s="3">
         <v>2</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="10" t="s">
         <v>671</v>
       </c>
       <c r="E56" s="6"/>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>54</v>
       </c>
@@ -4869,7 +4869,7 @@
       </c>
       <c r="E57" s="6"/>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>55</v>
       </c>
@@ -4879,12 +4879,12 @@
       <c r="C58" s="3">
         <v>1</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="10" t="s">
         <v>672</v>
       </c>
       <c r="E58" s="6"/>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>56</v>
       </c>
@@ -4894,12 +4894,12 @@
       <c r="C59" s="3">
         <v>1</v>
       </c>
-      <c r="D59" s="11" t="s">
+      <c r="D59" s="10" t="s">
         <v>672</v>
       </c>
       <c r="E59" s="6"/>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>57</v>
       </c>
@@ -4909,12 +4909,12 @@
       <c r="C60" s="3">
         <v>1</v>
       </c>
-      <c r="D60" s="11" t="s">
+      <c r="D60" s="10" t="s">
         <v>650</v>
       </c>
       <c r="E60" s="6"/>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="E61" s="6"/>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>59</v>
       </c>
@@ -4944,23 +4944,23 @@
       </c>
       <c r="E62" s="6"/>
     </row>
-    <row r="64" spans="1:5">
-      <c r="D64" s="11"/>
-    </row>
-    <row r="65" spans="4:4">
-      <c r="D65" s="12"/>
-    </row>
-    <row r="66" spans="4:4">
-      <c r="D66" s="11"/>
-    </row>
-    <row r="67" spans="4:4">
-      <c r="D67" s="13"/>
-    </row>
-    <row r="68" spans="4:4">
-      <c r="D68" s="12"/>
-    </row>
-    <row r="70" spans="4:4">
-      <c r="D70" s="12"/>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D64" s="10"/>
+    </row>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D65" s="11"/>
+    </row>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D66" s="10"/>
+    </row>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D68" s="11"/>
+    </row>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D70" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4971,7 +4971,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{396D6CEF-66BA-914C-BC20-42B24F721DE4}">
   <dimension ref="A1:I156"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.625" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
@@ -4982,7 +4982,7 @@
     <col min="9" max="9" width="33" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>67</v>
       </c>
@@ -5028,7 +5028,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>66</v>
       </c>
@@ -5045,7 +5045,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>116</v>
       </c>
@@ -5062,7 +5062,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>35</v>
       </c>
@@ -5079,7 +5079,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>34</v>
       </c>
@@ -5096,7 +5096,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
@@ -5148,7 +5148,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>130</v>
       </c>
@@ -5165,7 +5165,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>139</v>
       </c>
@@ -5182,7 +5182,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>140</v>
       </c>
@@ -5199,7 +5199,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>70</v>
       </c>
@@ -5216,7 +5216,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>76</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>68</v>
       </c>
@@ -5250,7 +5250,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>589</v>
       </c>
@@ -5264,7 +5264,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>52</v>
       </c>
@@ -5281,7 +5281,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>111</v>
       </c>
@@ -5298,7 +5298,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>110</v>
       </c>
@@ -5315,7 +5315,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>51</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>112</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>65</v>
       </c>
@@ -5366,7 +5366,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>86</v>
       </c>
@@ -5383,7 +5383,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>85</v>
       </c>
@@ -5400,7 +5400,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>97</v>
       </c>
@@ -5417,7 +5417,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>134</v>
       </c>
@@ -5434,7 +5434,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>133</v>
       </c>
@@ -5451,7 +5451,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>63</v>
       </c>
@@ -5468,7 +5468,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>91</v>
       </c>
@@ -5485,7 +5485,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>135</v>
       </c>
@@ -5502,7 +5502,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>113</v>
       </c>
@@ -5519,7 +5519,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>62</v>
       </c>
@@ -5536,7 +5536,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>64</v>
       </c>
@@ -5553,7 +5553,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>137</v>
       </c>
@@ -5570,7 +5570,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>455</v>
       </c>
@@ -5584,7 +5584,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>10</v>
       </c>
@@ -5610,7 +5610,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>32</v>
       </c>
@@ -5627,7 +5627,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>122</v>
       </c>
@@ -5644,7 +5644,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>120</v>
       </c>
@@ -5661,7 +5661,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>88</v>
       </c>
@@ -5678,7 +5678,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>129</v>
       </c>
@@ -5695,7 +5695,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>55</v>
       </c>
@@ -5712,7 +5712,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>56</v>
       </c>
@@ -5729,7 +5729,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>90</v>
       </c>
@@ -5746,7 +5746,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>33</v>
       </c>
@@ -5763,7 +5763,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>36</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>7</v>
       </c>
@@ -5806,7 +5806,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>9</v>
       </c>
@@ -5832,7 +5832,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>106</v>
       </c>
@@ -5849,7 +5849,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>593</v>
       </c>
@@ -5863,7 +5863,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>61</v>
       </c>
@@ -5880,7 +5880,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>107</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>98</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>93</v>
       </c>
@@ -5931,7 +5931,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>94</v>
       </c>
@@ -5948,7 +5948,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="55" spans="1:9">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>596</v>
       </c>
@@ -5962,7 +5962,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="56" spans="1:9">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>38</v>
       </c>
@@ -5979,7 +5979,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="57" spans="1:9">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>586</v>
       </c>
@@ -5993,7 +5993,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="58" spans="1:9">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>4</v>
       </c>
@@ -6019,7 +6019,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="59" spans="1:9">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>89</v>
       </c>
@@ -6036,7 +6036,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="60" spans="1:9">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>14</v>
       </c>
@@ -6062,7 +6062,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="61" spans="1:9">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>31</v>
       </c>
@@ -6079,7 +6079,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="62" spans="1:9">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>15</v>
       </c>
@@ -6105,7 +6105,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:9">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>108</v>
       </c>
@@ -6122,7 +6122,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="64" spans="1:9">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>21</v>
       </c>
@@ -6148,7 +6148,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="65" spans="1:9">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>123</v>
       </c>
@@ -6165,7 +6165,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="66" spans="1:9">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>602</v>
       </c>
@@ -6179,7 +6179,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="67" spans="1:9">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>60</v>
       </c>
@@ -6199,7 +6199,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="68" spans="1:9">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>25</v>
       </c>
@@ -6225,7 +6225,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>28</v>
       </c>
@@ -6251,7 +6251,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="70" spans="1:9">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>16</v>
       </c>
@@ -6277,7 +6277,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>26</v>
       </c>
@@ -6303,7 +6303,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>124</v>
       </c>
@@ -6320,7 +6320,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>104</v>
       </c>
@@ -6337,7 +6337,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="74" spans="1:9">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>125</v>
       </c>
@@ -6354,7 +6354,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="75" spans="1:9">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>109</v>
       </c>
@@ -6371,7 +6371,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="76" spans="1:9">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>29</v>
       </c>
@@ -6397,7 +6397,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="77" spans="1:9">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>141</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="78" spans="1:9">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
         <v>582</v>
       </c>
@@ -6428,7 +6428,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="79" spans="1:9">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>119</v>
       </c>
@@ -6445,7 +6445,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="80" spans="1:9">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>118</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
         <v>605</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>74</v>
       </c>
@@ -6493,7 +6493,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>75</v>
       </c>
@@ -6510,7 +6510,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>81</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>71</v>
       </c>
@@ -6544,7 +6544,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>73</v>
       </c>
@@ -6561,7 +6561,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>72</v>
       </c>
@@ -6578,7 +6578,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>80</v>
       </c>
@@ -6595,7 +6595,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>79</v>
       </c>
@@ -6612,7 +6612,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>69</v>
       </c>
@@ -6629,7 +6629,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>103</v>
       </c>
@@ -6646,7 +6646,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>102</v>
       </c>
@@ -6663,7 +6663,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>83</v>
       </c>
@@ -6680,7 +6680,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>82</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>84</v>
       </c>
@@ -6714,7 +6714,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>99</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>87</v>
       </c>
@@ -6748,7 +6748,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>126</v>
       </c>
@@ -6765,7 +6765,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="99" spans="1:9">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>12</v>
       </c>
@@ -6791,7 +6791,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="100" spans="1:9">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>5</v>
       </c>
@@ -6817,7 +6817,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="101" spans="1:9">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>127</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>39</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="103" spans="1:9">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>138</v>
       </c>
@@ -6871,7 +6871,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="104" spans="1:9">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>608</v>
       </c>
@@ -6885,7 +6885,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="105" spans="1:9">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>22</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="106" spans="1:9">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>30</v>
       </c>
@@ -6937,7 +6937,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="107" spans="1:9">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>17</v>
       </c>
@@ -6963,7 +6963,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="108" spans="1:9">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>19</v>
       </c>
@@ -6989,7 +6989,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:9">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>18</v>
       </c>
@@ -7015,7 +7015,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="110" spans="1:9">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>23</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="111" spans="1:9">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>128</v>
       </c>
@@ -7058,7 +7058,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="112" spans="1:9">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>95</v>
       </c>
@@ -7075,7 +7075,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="113" spans="1:9">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>101</v>
       </c>
@@ -7092,7 +7092,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="114" spans="1:9">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>100</v>
       </c>
@@ -7109,7 +7109,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="115" spans="1:9">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>105</v>
       </c>
@@ -7126,7 +7126,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="116" spans="1:9">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -7143,7 +7143,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="117" spans="1:9">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>131</v>
       </c>
@@ -7160,7 +7160,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="118" spans="1:9">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>20</v>
       </c>
@@ -7186,7 +7186,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="119" spans="1:9">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>13</v>
       </c>
@@ -7212,7 +7212,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="120" spans="1:9">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>24</v>
       </c>
@@ -7238,7 +7238,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="121" spans="1:9">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>132</v>
       </c>
@@ -7255,7 +7255,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="122" spans="1:9">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B122" t="s">
         <v>611</v>
       </c>
@@ -7269,7 +7269,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="123" spans="1:9">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B123" t="s">
         <v>599</v>
       </c>
@@ -7283,7 +7283,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="124" spans="1:9">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>1</v>
       </c>
@@ -7309,7 +7309,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="125" spans="1:9">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>8</v>
       </c>
@@ -7335,7 +7335,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="126" spans="1:9">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>6</v>
       </c>
@@ -7361,7 +7361,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="127" spans="1:9">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>11</v>
       </c>
@@ -7387,7 +7387,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="128" spans="1:9">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>27</v>
       </c>
@@ -7413,7 +7413,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="129" spans="1:7">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>121</v>
       </c>
@@ -7430,7 +7430,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="130" spans="1:7">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>54</v>
       </c>
@@ -7447,7 +7447,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="131" spans="1:7">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>53</v>
       </c>
@@ -7464,7 +7464,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>92</v>
       </c>
@@ -7481,7 +7481,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="133" spans="1:7">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
         <v>614</v>
       </c>
@@ -7495,7 +7495,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="134" spans="1:7">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>77</v>
       </c>
@@ -7512,7 +7512,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="135" spans="1:7">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>78</v>
       </c>
@@ -7529,7 +7529,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="136" spans="1:7">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>46</v>
       </c>
@@ -7546,7 +7546,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="137" spans="1:7">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>43</v>
       </c>
@@ -7563,7 +7563,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="138" spans="1:7">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>45</v>
       </c>
@@ -7580,7 +7580,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="139" spans="1:7">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>42</v>
       </c>
@@ -7597,7 +7597,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="140" spans="1:7">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>50</v>
       </c>
@@ -7614,7 +7614,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="141" spans="1:7">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>49</v>
       </c>
@@ -7631,7 +7631,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="142" spans="1:7">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>44</v>
       </c>
@@ -7648,7 +7648,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="143" spans="1:7">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>41</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="144" spans="1:7">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>40</v>
       </c>
@@ -7682,7 +7682,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="145" spans="1:7">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>37</v>
       </c>
@@ -7699,7 +7699,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="146" spans="1:7">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>48</v>
       </c>
@@ -7716,7 +7716,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="147" spans="1:7">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>114</v>
       </c>
@@ -7733,7 +7733,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="148" spans="1:7">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>47</v>
       </c>
@@ -7750,7 +7750,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="149" spans="1:7">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>544</v>
       </c>
@@ -7764,7 +7764,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="150" spans="1:7">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>117</v>
       </c>
@@ -7781,7 +7781,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="151" spans="1:7">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>96</v>
       </c>
@@ -7798,7 +7798,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="152" spans="1:7">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B152" t="s">
         <v>547</v>
       </c>
@@ -7812,7 +7812,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="153" spans="1:7">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>57</v>
       </c>
@@ -7829,7 +7829,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="154" spans="1:7">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>59</v>
       </c>
@@ -7846,7 +7846,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="155" spans="1:7">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>58</v>
       </c>
@@ -7863,7 +7863,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="156" spans="1:7">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>136</v>
       </c>

</xml_diff>